<commit_message>
Questions tab: three slots per section, one column per vendor
Replaces the shared tick-list with a vendor-specific grid: the six
questionnaire sections each hold three question rows across twenty vendor
columns. The first sixteen headers follow the names typed on the Scorecard.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119SWLvpPHQDhSpwCbaRpx4
</commit_message>
<xml_diff>
--- a/agents/compassus-capacity-pm/vendor-evaluation/Vendor-Scorecard.xlsx
+++ b/agents/compassus-capacity-pm/vendor-evaluation/Vendor-Scorecard.xlsx
@@ -21,6 +21,7 @@
     <definedName name="Part_List">Lists!$K$2:$K$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Example'!$5:$10,'Example'!$B:$E</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scorecard'!$5:$10,'Scorecard'!$B:$E</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Questions'!$5:$5,'Questions'!$B:$C</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +32,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -198,12 +199,6 @@
       <color rgb="00792E2E"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color rgb="001B211E"/>
-      <sz val="18"/>
-    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -342,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -520,21 +515,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7609,1338 +7594,648 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:X66"/>
+  <dimension ref="B2:W35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="74" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="15" customWidth="1" min="23" max="23"/>
-    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="34" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="52" t="inlineStr">
-        <is>
-          <t>COMPASSUS  ·  HOME HEALTH</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
-      <c r="B3" s="63" t="inlineStr">
-        <is>
-          <t>Follow-up Questions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>What we make them prove at the demo. Written as the returns come in, in the order the questionnaire asks — so a gap found while scoring lands next to the question that exposed it. Mark the vendors each one applies to.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>VENDOR</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 01</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 02</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 03</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 04</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 05</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 06</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 07</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 08</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 09</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 10</t>
-        </is>
-      </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 11</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 12</t>
-        </is>
-      </c>
-      <c r="Q6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 13</t>
-        </is>
-      </c>
-      <c r="R6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 14</t>
-        </is>
-      </c>
-      <c r="S6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 15</t>
-        </is>
-      </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>Vendor 16</t>
-        </is>
-      </c>
-      <c r="U6" s="6" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>COMPASSUS  ·  CAPACITY &amp; SCHEDULING</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>What we make each vendor prove at the demo. Three per section, written as the return is scored, so a gap lands next to the question that exposed it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D5" s="6">
+        <f>IF(Scorecard!F5="","Vendor 01",Scorecard!F5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>IF(Scorecard!H5="","Vendor 02",Scorecard!H5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>IF(Scorecard!J5="","Vendor 03",Scorecard!J5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="6">
+        <f>IF(Scorecard!L5="","Vendor 04",Scorecard!L5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="6">
+        <f>IF(Scorecard!N5="","Vendor 05",Scorecard!N5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
+        <f>IF(Scorecard!P5="","Vendor 06",Scorecard!P5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>IF(Scorecard!R5="","Vendor 07",Scorecard!R5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="6">
+        <f>IF(Scorecard!T5="","Vendor 08",Scorecard!T5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>IF(Scorecard!V5="","Vendor 09",Scorecard!V5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="6">
+        <f>IF(Scorecard!X5="","Vendor 10",Scorecard!X5)</f>
+        <v/>
+      </c>
+      <c r="N5" s="6">
+        <f>IF(Scorecard!Z5="","Vendor 11",Scorecard!Z5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="6">
+        <f>IF(Scorecard!AB5="","Vendor 12",Scorecard!AB5)</f>
+        <v/>
+      </c>
+      <c r="P5" s="6">
+        <f>IF(Scorecard!AD5="","Vendor 13",Scorecard!AD5)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="6">
+        <f>IF(Scorecard!AF5="","Vendor 14",Scorecard!AF5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="6">
+        <f>IF(Scorecard!AH5="","Vendor 15",Scorecard!AH5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="6">
+        <f>IF(Scorecard!AJ5="","Vendor 16",Scorecard!AJ5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="6" t="inlineStr">
         <is>
           <t>Vendor 17</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>Vendor 18</t>
         </is>
       </c>
-      <c r="W6" s="6" t="inlineStr">
+      <c r="V5" s="6" t="inlineStr">
         <is>
           <t>Vendor 19</t>
         </is>
       </c>
-      <c r="X6" s="6" t="inlineStr">
+      <c r="W5" s="6" t="inlineStr">
         <is>
           <t>Vendor 20</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="21" customHeight="1">
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>A  ·  COMPANY AND PRODUCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>A1 integration · A2 scale and references · A3 measured impact</t>
-        </is>
-      </c>
-      <c r="D9" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="65" t="n"/>
-      <c r="C10" s="66" t="n"/>
-      <c r="D10" s="67" t="n"/>
-      <c r="E10" s="68" t="n"/>
-      <c r="F10" s="68" t="n"/>
-      <c r="G10" s="68" t="n"/>
-      <c r="H10" s="68" t="n"/>
-      <c r="I10" s="68" t="n"/>
-      <c r="J10" s="68" t="n"/>
-      <c r="K10" s="68" t="n"/>
-      <c r="L10" s="68" t="n"/>
-      <c r="M10" s="68" t="n"/>
-      <c r="N10" s="68" t="n"/>
-      <c r="O10" s="68" t="n"/>
-      <c r="P10" s="68" t="n"/>
-      <c r="Q10" s="68" t="n"/>
-      <c r="R10" s="68" t="n"/>
-      <c r="S10" s="68" t="n"/>
-      <c r="T10" s="68" t="n"/>
-      <c r="U10" s="68" t="n"/>
-      <c r="V10" s="68" t="n"/>
-      <c r="W10" s="68" t="n"/>
-      <c r="X10" s="68" t="n"/>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="65" t="n"/>
-      <c r="C11" s="66" t="n"/>
-      <c r="D11" s="67" t="n"/>
-      <c r="E11" s="68" t="n"/>
-      <c r="F11" s="68" t="n"/>
-      <c r="G11" s="68" t="n"/>
-      <c r="H11" s="68" t="n"/>
-      <c r="I11" s="68" t="n"/>
-      <c r="J11" s="68" t="n"/>
-      <c r="K11" s="68" t="n"/>
-      <c r="L11" s="68" t="n"/>
-      <c r="M11" s="68" t="n"/>
-      <c r="N11" s="68" t="n"/>
-      <c r="O11" s="68" t="n"/>
-      <c r="P11" s="68" t="n"/>
-      <c r="Q11" s="68" t="n"/>
-      <c r="R11" s="68" t="n"/>
-      <c r="S11" s="68" t="n"/>
-      <c r="T11" s="68" t="n"/>
-      <c r="U11" s="68" t="n"/>
-      <c r="V11" s="68" t="n"/>
-      <c r="W11" s="68" t="n"/>
-      <c r="X11" s="68" t="n"/>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="B12" s="65" t="n"/>
-      <c r="C12" s="66" t="n"/>
-      <c r="D12" s="67" t="n"/>
-      <c r="E12" s="68" t="n"/>
-      <c r="F12" s="68" t="n"/>
-      <c r="G12" s="68" t="n"/>
-      <c r="H12" s="68" t="n"/>
-      <c r="I12" s="68" t="n"/>
-      <c r="J12" s="68" t="n"/>
-      <c r="K12" s="68" t="n"/>
-      <c r="L12" s="68" t="n"/>
-      <c r="M12" s="68" t="n"/>
-      <c r="N12" s="68" t="n"/>
-      <c r="O12" s="68" t="n"/>
-      <c r="P12" s="68" t="n"/>
-      <c r="Q12" s="68" t="n"/>
-      <c r="R12" s="68" t="n"/>
-      <c r="S12" s="68" t="n"/>
-      <c r="T12" s="68" t="n"/>
-      <c r="U12" s="68" t="n"/>
-      <c r="V12" s="68" t="n"/>
-      <c r="W12" s="68" t="n"/>
-      <c r="X12" s="68" t="n"/>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="65" t="n"/>
-      <c r="C13" s="66" t="n"/>
-      <c r="D13" s="67" t="n"/>
-      <c r="E13" s="68" t="n"/>
-      <c r="F13" s="68" t="n"/>
-      <c r="G13" s="68" t="n"/>
-      <c r="H13" s="68" t="n"/>
-      <c r="I13" s="68" t="n"/>
-      <c r="J13" s="68" t="n"/>
-      <c r="K13" s="68" t="n"/>
-      <c r="L13" s="68" t="n"/>
-      <c r="M13" s="68" t="n"/>
-      <c r="N13" s="68" t="n"/>
-      <c r="O13" s="68" t="n"/>
-      <c r="P13" s="68" t="n"/>
-      <c r="Q13" s="68" t="n"/>
-      <c r="R13" s="68" t="n"/>
-      <c r="S13" s="68" t="n"/>
-      <c r="T13" s="68" t="n"/>
-      <c r="U13" s="68" t="n"/>
-      <c r="V13" s="68" t="n"/>
-      <c r="W13" s="68" t="n"/>
-      <c r="X13" s="68" t="n"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="B14" s="65" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="68" t="n"/>
-      <c r="G14" s="68" t="n"/>
-      <c r="H14" s="68" t="n"/>
-      <c r="I14" s="68" t="n"/>
-      <c r="J14" s="68" t="n"/>
-      <c r="K14" s="68" t="n"/>
-      <c r="L14" s="68" t="n"/>
-      <c r="M14" s="68" t="n"/>
-      <c r="N14" s="68" t="n"/>
-      <c r="O14" s="68" t="n"/>
-      <c r="P14" s="68" t="n"/>
-      <c r="Q14" s="68" t="n"/>
-      <c r="R14" s="68" t="n"/>
-      <c r="S14" s="68" t="n"/>
-      <c r="T14" s="68" t="n"/>
-      <c r="U14" s="68" t="n"/>
-      <c r="V14" s="68" t="n"/>
-      <c r="W14" s="68" t="n"/>
-      <c r="X14" s="68" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="65" t="n"/>
-      <c r="C15" s="66" t="n"/>
-      <c r="D15" s="67" t="n"/>
-      <c r="E15" s="68" t="n"/>
-      <c r="F15" s="68" t="n"/>
-      <c r="G15" s="68" t="n"/>
-      <c r="H15" s="68" t="n"/>
-      <c r="I15" s="68" t="n"/>
-      <c r="J15" s="68" t="n"/>
-      <c r="K15" s="68" t="n"/>
-      <c r="L15" s="68" t="n"/>
-      <c r="M15" s="68" t="n"/>
-      <c r="N15" s="68" t="n"/>
-      <c r="O15" s="68" t="n"/>
-      <c r="P15" s="68" t="n"/>
-      <c r="Q15" s="68" t="n"/>
-      <c r="R15" s="68" t="n"/>
-      <c r="S15" s="68" t="n"/>
-      <c r="T15" s="68" t="n"/>
-      <c r="U15" s="68" t="n"/>
-      <c r="V15" s="68" t="n"/>
-      <c r="W15" s="68" t="n"/>
-      <c r="X15" s="68" t="n"/>
+    <row r="7" ht="21" customHeight="1">
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>A  ·  COMPANY AND PRODUCT      A1 integration · A2 scale and references · A3 measured impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="B8" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="64" t="n"/>
+      <c r="E8" s="64" t="n"/>
+      <c r="F8" s="64" t="n"/>
+      <c r="G8" s="64" t="n"/>
+      <c r="H8" s="64" t="n"/>
+      <c r="I8" s="64" t="n"/>
+      <c r="J8" s="64" t="n"/>
+      <c r="K8" s="64" t="n"/>
+      <c r="L8" s="64" t="n"/>
+      <c r="M8" s="64" t="n"/>
+      <c r="N8" s="64" t="n"/>
+      <c r="O8" s="64" t="n"/>
+      <c r="P8" s="64" t="n"/>
+      <c r="Q8" s="64" t="n"/>
+      <c r="R8" s="64" t="n"/>
+      <c r="S8" s="64" t="n"/>
+      <c r="T8" s="64" t="n"/>
+      <c r="U8" s="64" t="n"/>
+      <c r="V8" s="64" t="n"/>
+      <c r="W8" s="64" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="B9" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="64" t="n"/>
+      <c r="E9" s="64" t="n"/>
+      <c r="F9" s="64" t="n"/>
+      <c r="G9" s="64" t="n"/>
+      <c r="H9" s="64" t="n"/>
+      <c r="I9" s="64" t="n"/>
+      <c r="J9" s="64" t="n"/>
+      <c r="K9" s="64" t="n"/>
+      <c r="L9" s="64" t="n"/>
+      <c r="M9" s="64" t="n"/>
+      <c r="N9" s="64" t="n"/>
+      <c r="O9" s="64" t="n"/>
+      <c r="P9" s="64" t="n"/>
+      <c r="Q9" s="64" t="n"/>
+      <c r="R9" s="64" t="n"/>
+      <c r="S9" s="64" t="n"/>
+      <c r="T9" s="64" t="n"/>
+      <c r="U9" s="64" t="n"/>
+      <c r="V9" s="64" t="n"/>
+      <c r="W9" s="64" t="n"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="B10" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="64" t="n"/>
+      <c r="E10" s="64" t="n"/>
+      <c r="F10" s="64" t="n"/>
+      <c r="G10" s="64" t="n"/>
+      <c r="H10" s="64" t="n"/>
+      <c r="I10" s="64" t="n"/>
+      <c r="J10" s="64" t="n"/>
+      <c r="K10" s="64" t="n"/>
+      <c r="L10" s="64" t="n"/>
+      <c r="M10" s="64" t="n"/>
+      <c r="N10" s="64" t="n"/>
+      <c r="O10" s="64" t="n"/>
+      <c r="P10" s="64" t="n"/>
+      <c r="Q10" s="64" t="n"/>
+      <c r="R10" s="64" t="n"/>
+      <c r="S10" s="64" t="n"/>
+      <c r="T10" s="64" t="n"/>
+      <c r="U10" s="64" t="n"/>
+      <c r="V10" s="64" t="n"/>
+      <c r="W10" s="64" t="n"/>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>B  ·  COVERAGE SELF-ASSESSMENT      anything claimed in scope that Section C did not support</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="B13" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="64" t="n"/>
+      <c r="E13" s="64" t="n"/>
+      <c r="F13" s="64" t="n"/>
+      <c r="G13" s="64" t="n"/>
+      <c r="H13" s="64" t="n"/>
+      <c r="I13" s="64" t="n"/>
+      <c r="J13" s="64" t="n"/>
+      <c r="K13" s="64" t="n"/>
+      <c r="L13" s="64" t="n"/>
+      <c r="M13" s="64" t="n"/>
+      <c r="N13" s="64" t="n"/>
+      <c r="O13" s="64" t="n"/>
+      <c r="P13" s="64" t="n"/>
+      <c r="Q13" s="64" t="n"/>
+      <c r="R13" s="64" t="n"/>
+      <c r="S13" s="64" t="n"/>
+      <c r="T13" s="64" t="n"/>
+      <c r="U13" s="64" t="n"/>
+      <c r="V13" s="64" t="n"/>
+      <c r="W13" s="64" t="n"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="B14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="64" t="n"/>
+      <c r="E14" s="64" t="n"/>
+      <c r="F14" s="64" t="n"/>
+      <c r="G14" s="64" t="n"/>
+      <c r="H14" s="64" t="n"/>
+      <c r="I14" s="64" t="n"/>
+      <c r="J14" s="64" t="n"/>
+      <c r="K14" s="64" t="n"/>
+      <c r="L14" s="64" t="n"/>
+      <c r="M14" s="64" t="n"/>
+      <c r="N14" s="64" t="n"/>
+      <c r="O14" s="64" t="n"/>
+      <c r="P14" s="64" t="n"/>
+      <c r="Q14" s="64" t="n"/>
+      <c r="R14" s="64" t="n"/>
+      <c r="S14" s="64" t="n"/>
+      <c r="T14" s="64" t="n"/>
+      <c r="U14" s="64" t="n"/>
+      <c r="V14" s="64" t="n"/>
+      <c r="W14" s="64" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="B15" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="64" t="n"/>
+      <c r="E15" s="64" t="n"/>
+      <c r="F15" s="64" t="n"/>
+      <c r="G15" s="64" t="n"/>
+      <c r="H15" s="64" t="n"/>
+      <c r="I15" s="64" t="n"/>
+      <c r="J15" s="64" t="n"/>
+      <c r="K15" s="64" t="n"/>
+      <c r="L15" s="64" t="n"/>
+      <c r="M15" s="64" t="n"/>
+      <c r="N15" s="64" t="n"/>
+      <c r="O15" s="64" t="n"/>
+      <c r="P15" s="64" t="n"/>
+      <c r="Q15" s="64" t="n"/>
+      <c r="R15" s="64" t="n"/>
+      <c r="S15" s="64" t="n"/>
+      <c r="T15" s="64" t="n"/>
+      <c r="U15" s="64" t="n"/>
+      <c r="V15" s="64" t="n"/>
+      <c r="W15" s="64" t="n"/>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>B  ·  COVERAGE SELF-ASSESSMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Anything they claimed in scope that Section C did not support</t>
-        </is>
-      </c>
-      <c r="D18" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="65" t="n"/>
-      <c r="C19" s="66" t="n"/>
-      <c r="D19" s="67" t="n"/>
-      <c r="E19" s="68" t="n"/>
-      <c r="F19" s="68" t="n"/>
-      <c r="G19" s="68" t="n"/>
-      <c r="H19" s="68" t="n"/>
-      <c r="I19" s="68" t="n"/>
-      <c r="J19" s="68" t="n"/>
-      <c r="K19" s="68" t="n"/>
-      <c r="L19" s="68" t="n"/>
-      <c r="M19" s="68" t="n"/>
-      <c r="N19" s="68" t="n"/>
-      <c r="O19" s="68" t="n"/>
-      <c r="P19" s="68" t="n"/>
-      <c r="Q19" s="68" t="n"/>
-      <c r="R19" s="68" t="n"/>
-      <c r="S19" s="68" t="n"/>
-      <c r="T19" s="68" t="n"/>
-      <c r="U19" s="68" t="n"/>
-      <c r="V19" s="68" t="n"/>
-      <c r="W19" s="68" t="n"/>
-      <c r="X19" s="68" t="n"/>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="B20" s="65" t="n"/>
-      <c r="C20" s="66" t="n"/>
-      <c r="D20" s="67" t="n"/>
-      <c r="E20" s="68" t="n"/>
-      <c r="F20" s="68" t="n"/>
-      <c r="G20" s="68" t="n"/>
-      <c r="H20" s="68" t="n"/>
-      <c r="I20" s="68" t="n"/>
-      <c r="J20" s="68" t="n"/>
-      <c r="K20" s="68" t="n"/>
-      <c r="L20" s="68" t="n"/>
-      <c r="M20" s="68" t="n"/>
-      <c r="N20" s="68" t="n"/>
-      <c r="O20" s="68" t="n"/>
-      <c r="P20" s="68" t="n"/>
-      <c r="Q20" s="68" t="n"/>
-      <c r="R20" s="68" t="n"/>
-      <c r="S20" s="68" t="n"/>
-      <c r="T20" s="68" t="n"/>
-      <c r="U20" s="68" t="n"/>
-      <c r="V20" s="68" t="n"/>
-      <c r="W20" s="68" t="n"/>
-      <c r="X20" s="68" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="65" t="n"/>
-      <c r="C21" s="66" t="n"/>
-      <c r="D21" s="67" t="n"/>
-      <c r="E21" s="68" t="n"/>
-      <c r="F21" s="68" t="n"/>
-      <c r="G21" s="68" t="n"/>
-      <c r="H21" s="68" t="n"/>
-      <c r="I21" s="68" t="n"/>
-      <c r="J21" s="68" t="n"/>
-      <c r="K21" s="68" t="n"/>
-      <c r="L21" s="68" t="n"/>
-      <c r="M21" s="68" t="n"/>
-      <c r="N21" s="68" t="n"/>
-      <c r="O21" s="68" t="n"/>
-      <c r="P21" s="68" t="n"/>
-      <c r="Q21" s="68" t="n"/>
-      <c r="R21" s="68" t="n"/>
-      <c r="S21" s="68" t="n"/>
-      <c r="T21" s="68" t="n"/>
-      <c r="U21" s="68" t="n"/>
-      <c r="V21" s="68" t="n"/>
-      <c r="W21" s="68" t="n"/>
-      <c r="X21" s="68" t="n"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="B22" s="65" t="n"/>
-      <c r="C22" s="66" t="n"/>
-      <c r="D22" s="67" t="n"/>
-      <c r="E22" s="68" t="n"/>
-      <c r="F22" s="68" t="n"/>
-      <c r="G22" s="68" t="n"/>
-      <c r="H22" s="68" t="n"/>
-      <c r="I22" s="68" t="n"/>
-      <c r="J22" s="68" t="n"/>
-      <c r="K22" s="68" t="n"/>
-      <c r="L22" s="68" t="n"/>
-      <c r="M22" s="68" t="n"/>
-      <c r="N22" s="68" t="n"/>
-      <c r="O22" s="68" t="n"/>
-      <c r="P22" s="68" t="n"/>
-      <c r="Q22" s="68" t="n"/>
-      <c r="R22" s="68" t="n"/>
-      <c r="S22" s="68" t="n"/>
-      <c r="T22" s="68" t="n"/>
-      <c r="U22" s="68" t="n"/>
-      <c r="V22" s="68" t="n"/>
-      <c r="W22" s="68" t="n"/>
-      <c r="X22" s="68" t="n"/>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="65" t="n"/>
-      <c r="C23" s="66" t="n"/>
-      <c r="D23" s="67" t="n"/>
-      <c r="E23" s="68" t="n"/>
-      <c r="F23" s="68" t="n"/>
-      <c r="G23" s="68" t="n"/>
-      <c r="H23" s="68" t="n"/>
-      <c r="I23" s="68" t="n"/>
-      <c r="J23" s="68" t="n"/>
-      <c r="K23" s="68" t="n"/>
-      <c r="L23" s="68" t="n"/>
-      <c r="M23" s="68" t="n"/>
-      <c r="N23" s="68" t="n"/>
-      <c r="O23" s="68" t="n"/>
-      <c r="P23" s="68" t="n"/>
-      <c r="Q23" s="68" t="n"/>
-      <c r="R23" s="68" t="n"/>
-      <c r="S23" s="68" t="n"/>
-      <c r="T23" s="68" t="n"/>
-      <c r="U23" s="68" t="n"/>
-      <c r="V23" s="68" t="n"/>
-      <c r="W23" s="68" t="n"/>
-      <c r="X23" s="68" t="n"/>
-    </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="65" t="n"/>
-      <c r="C24" s="66" t="n"/>
-      <c r="D24" s="67" t="n"/>
-      <c r="E24" s="68" t="n"/>
-      <c r="F24" s="68" t="n"/>
-      <c r="G24" s="68" t="n"/>
-      <c r="H24" s="68" t="n"/>
-      <c r="I24" s="68" t="n"/>
-      <c r="J24" s="68" t="n"/>
-      <c r="K24" s="68" t="n"/>
-      <c r="L24" s="68" t="n"/>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="68" t="n"/>
-      <c r="O24" s="68" t="n"/>
-      <c r="P24" s="68" t="n"/>
-      <c r="Q24" s="68" t="n"/>
-      <c r="R24" s="68" t="n"/>
-      <c r="S24" s="68" t="n"/>
-      <c r="T24" s="68" t="n"/>
-      <c r="U24" s="68" t="n"/>
-      <c r="V24" s="68" t="n"/>
-      <c r="W24" s="68" t="n"/>
-      <c r="X24" s="68" t="n"/>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="65" t="n"/>
-      <c r="C25" s="66" t="n"/>
-      <c r="D25" s="67" t="n"/>
-      <c r="E25" s="68" t="n"/>
-      <c r="F25" s="68" t="n"/>
-      <c r="G25" s="68" t="n"/>
-      <c r="H25" s="68" t="n"/>
-      <c r="I25" s="68" t="n"/>
-      <c r="J25" s="68" t="n"/>
-      <c r="K25" s="68" t="n"/>
-      <c r="L25" s="68" t="n"/>
-      <c r="M25" s="68" t="n"/>
-      <c r="N25" s="68" t="n"/>
-      <c r="O25" s="68" t="n"/>
-      <c r="P25" s="68" t="n"/>
-      <c r="Q25" s="68" t="n"/>
-      <c r="R25" s="68" t="n"/>
-      <c r="S25" s="68" t="n"/>
-      <c r="T25" s="68" t="n"/>
-      <c r="U25" s="68" t="n"/>
-      <c r="V25" s="68" t="n"/>
-      <c r="W25" s="68" t="n"/>
-      <c r="X25" s="68" t="n"/>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="65" t="n"/>
-      <c r="C26" s="66" t="n"/>
-      <c r="D26" s="67" t="n"/>
-      <c r="E26" s="68" t="n"/>
-      <c r="F26" s="68" t="n"/>
-      <c r="G26" s="68" t="n"/>
-      <c r="H26" s="68" t="n"/>
-      <c r="I26" s="68" t="n"/>
-      <c r="J26" s="68" t="n"/>
-      <c r="K26" s="68" t="n"/>
-      <c r="L26" s="68" t="n"/>
-      <c r="M26" s="68" t="n"/>
-      <c r="N26" s="68" t="n"/>
-      <c r="O26" s="68" t="n"/>
-      <c r="P26" s="68" t="n"/>
-      <c r="Q26" s="68" t="n"/>
-      <c r="R26" s="68" t="n"/>
-      <c r="S26" s="68" t="n"/>
-      <c r="T26" s="68" t="n"/>
-      <c r="U26" s="68" t="n"/>
-      <c r="V26" s="68" t="n"/>
-      <c r="W26" s="68" t="n"/>
-      <c r="X26" s="68" t="n"/>
-    </row>
-    <row r="28" ht="21" customHeight="1">
-      <c r="B28" s="27" t="inlineStr">
-        <is>
-          <t>C  ·  HOW YOUR PRODUCT WORKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>C1 capacity · C2 assignment · C3 readiness · C4 the week · C5 recovery · C6 downtime · C7 the patient</t>
-        </is>
-      </c>
-      <c r="D29" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="65" t="n"/>
-      <c r="C30" s="66" t="n"/>
-      <c r="D30" s="67" t="n"/>
-      <c r="E30" s="68" t="n"/>
-      <c r="F30" s="68" t="n"/>
-      <c r="G30" s="68" t="n"/>
-      <c r="H30" s="68" t="n"/>
-      <c r="I30" s="68" t="n"/>
-      <c r="J30" s="68" t="n"/>
-      <c r="K30" s="68" t="n"/>
-      <c r="L30" s="68" t="n"/>
-      <c r="M30" s="68" t="n"/>
-      <c r="N30" s="68" t="n"/>
-      <c r="O30" s="68" t="n"/>
-      <c r="P30" s="68" t="n"/>
-      <c r="Q30" s="68" t="n"/>
-      <c r="R30" s="68" t="n"/>
-      <c r="S30" s="68" t="n"/>
-      <c r="T30" s="68" t="n"/>
-      <c r="U30" s="68" t="n"/>
-      <c r="V30" s="68" t="n"/>
-      <c r="W30" s="68" t="n"/>
-      <c r="X30" s="68" t="n"/>
-    </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="65" t="n"/>
-      <c r="C31" s="66" t="n"/>
-      <c r="D31" s="67" t="n"/>
-      <c r="E31" s="68" t="n"/>
-      <c r="F31" s="68" t="n"/>
-      <c r="G31" s="68" t="n"/>
-      <c r="H31" s="68" t="n"/>
-      <c r="I31" s="68" t="n"/>
-      <c r="J31" s="68" t="n"/>
-      <c r="K31" s="68" t="n"/>
-      <c r="L31" s="68" t="n"/>
-      <c r="M31" s="68" t="n"/>
-      <c r="N31" s="68" t="n"/>
-      <c r="O31" s="68" t="n"/>
-      <c r="P31" s="68" t="n"/>
-      <c r="Q31" s="68" t="n"/>
-      <c r="R31" s="68" t="n"/>
-      <c r="S31" s="68" t="n"/>
-      <c r="T31" s="68" t="n"/>
-      <c r="U31" s="68" t="n"/>
-      <c r="V31" s="68" t="n"/>
-      <c r="W31" s="68" t="n"/>
-      <c r="X31" s="68" t="n"/>
-    </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="65" t="n"/>
-      <c r="C32" s="66" t="n"/>
-      <c r="D32" s="67" t="n"/>
-      <c r="E32" s="68" t="n"/>
-      <c r="F32" s="68" t="n"/>
-      <c r="G32" s="68" t="n"/>
-      <c r="H32" s="68" t="n"/>
-      <c r="I32" s="68" t="n"/>
-      <c r="J32" s="68" t="n"/>
-      <c r="K32" s="68" t="n"/>
-      <c r="L32" s="68" t="n"/>
-      <c r="M32" s="68" t="n"/>
-      <c r="N32" s="68" t="n"/>
-      <c r="O32" s="68" t="n"/>
-      <c r="P32" s="68" t="n"/>
-      <c r="Q32" s="68" t="n"/>
-      <c r="R32" s="68" t="n"/>
-      <c r="S32" s="68" t="n"/>
-      <c r="T32" s="68" t="n"/>
-      <c r="U32" s="68" t="n"/>
-      <c r="V32" s="68" t="n"/>
-      <c r="W32" s="68" t="n"/>
-      <c r="X32" s="68" t="n"/>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="65" t="n"/>
-      <c r="C33" s="66" t="n"/>
-      <c r="D33" s="67" t="n"/>
-      <c r="E33" s="68" t="n"/>
-      <c r="F33" s="68" t="n"/>
-      <c r="G33" s="68" t="n"/>
-      <c r="H33" s="68" t="n"/>
-      <c r="I33" s="68" t="n"/>
-      <c r="J33" s="68" t="n"/>
-      <c r="K33" s="68" t="n"/>
-      <c r="L33" s="68" t="n"/>
-      <c r="M33" s="68" t="n"/>
-      <c r="N33" s="68" t="n"/>
-      <c r="O33" s="68" t="n"/>
-      <c r="P33" s="68" t="n"/>
-      <c r="Q33" s="68" t="n"/>
-      <c r="R33" s="68" t="n"/>
-      <c r="S33" s="68" t="n"/>
-      <c r="T33" s="68" t="n"/>
-      <c r="U33" s="68" t="n"/>
-      <c r="V33" s="68" t="n"/>
-      <c r="W33" s="68" t="n"/>
-      <c r="X33" s="68" t="n"/>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="B34" s="65" t="n"/>
-      <c r="C34" s="66" t="n"/>
-      <c r="D34" s="67" t="n"/>
-      <c r="E34" s="68" t="n"/>
-      <c r="F34" s="68" t="n"/>
-      <c r="G34" s="68" t="n"/>
-      <c r="H34" s="68" t="n"/>
-      <c r="I34" s="68" t="n"/>
-      <c r="J34" s="68" t="n"/>
-      <c r="K34" s="68" t="n"/>
-      <c r="L34" s="68" t="n"/>
-      <c r="M34" s="68" t="n"/>
-      <c r="N34" s="68" t="n"/>
-      <c r="O34" s="68" t="n"/>
-      <c r="P34" s="68" t="n"/>
-      <c r="Q34" s="68" t="n"/>
-      <c r="R34" s="68" t="n"/>
-      <c r="S34" s="68" t="n"/>
-      <c r="T34" s="68" t="n"/>
-      <c r="U34" s="68" t="n"/>
-      <c r="V34" s="68" t="n"/>
-      <c r="W34" s="68" t="n"/>
-      <c r="X34" s="68" t="n"/>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="65" t="n"/>
-      <c r="C35" s="66" t="n"/>
-      <c r="D35" s="67" t="n"/>
-      <c r="E35" s="68" t="n"/>
-      <c r="F35" s="68" t="n"/>
-      <c r="G35" s="68" t="n"/>
-      <c r="H35" s="68" t="n"/>
-      <c r="I35" s="68" t="n"/>
-      <c r="J35" s="68" t="n"/>
-      <c r="K35" s="68" t="n"/>
-      <c r="L35" s="68" t="n"/>
-      <c r="M35" s="68" t="n"/>
-      <c r="N35" s="68" t="n"/>
-      <c r="O35" s="68" t="n"/>
-      <c r="P35" s="68" t="n"/>
-      <c r="Q35" s="68" t="n"/>
-      <c r="R35" s="68" t="n"/>
-      <c r="S35" s="68" t="n"/>
-      <c r="T35" s="68" t="n"/>
-      <c r="U35" s="68" t="n"/>
-      <c r="V35" s="68" t="n"/>
-      <c r="W35" s="68" t="n"/>
-      <c r="X35" s="68" t="n"/>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="B36" s="65" t="n"/>
-      <c r="C36" s="66" t="n"/>
-      <c r="D36" s="67" t="n"/>
-      <c r="E36" s="68" t="n"/>
-      <c r="F36" s="68" t="n"/>
-      <c r="G36" s="68" t="n"/>
-      <c r="H36" s="68" t="n"/>
-      <c r="I36" s="68" t="n"/>
-      <c r="J36" s="68" t="n"/>
-      <c r="K36" s="68" t="n"/>
-      <c r="L36" s="68" t="n"/>
-      <c r="M36" s="68" t="n"/>
-      <c r="N36" s="68" t="n"/>
-      <c r="O36" s="68" t="n"/>
-      <c r="P36" s="68" t="n"/>
-      <c r="Q36" s="68" t="n"/>
-      <c r="R36" s="68" t="n"/>
-      <c r="S36" s="68" t="n"/>
-      <c r="T36" s="68" t="n"/>
-      <c r="U36" s="68" t="n"/>
-      <c r="V36" s="68" t="n"/>
-      <c r="W36" s="68" t="n"/>
-      <c r="X36" s="68" t="n"/>
-    </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="B37" s="65" t="n"/>
-      <c r="C37" s="66" t="n"/>
-      <c r="D37" s="67" t="n"/>
-      <c r="E37" s="68" t="n"/>
-      <c r="F37" s="68" t="n"/>
-      <c r="G37" s="68" t="n"/>
-      <c r="H37" s="68" t="n"/>
-      <c r="I37" s="68" t="n"/>
-      <c r="J37" s="68" t="n"/>
-      <c r="K37" s="68" t="n"/>
-      <c r="L37" s="68" t="n"/>
-      <c r="M37" s="68" t="n"/>
-      <c r="N37" s="68" t="n"/>
-      <c r="O37" s="68" t="n"/>
-      <c r="P37" s="68" t="n"/>
-      <c r="Q37" s="68" t="n"/>
-      <c r="R37" s="68" t="n"/>
-      <c r="S37" s="68" t="n"/>
-      <c r="T37" s="68" t="n"/>
-      <c r="U37" s="68" t="n"/>
-      <c r="V37" s="68" t="n"/>
-      <c r="W37" s="68" t="n"/>
-      <c r="X37" s="68" t="n"/>
-    </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="B38" s="65" t="n"/>
-      <c r="C38" s="66" t="n"/>
-      <c r="D38" s="67" t="n"/>
-      <c r="E38" s="68" t="n"/>
-      <c r="F38" s="68" t="n"/>
-      <c r="G38" s="68" t="n"/>
-      <c r="H38" s="68" t="n"/>
-      <c r="I38" s="68" t="n"/>
-      <c r="J38" s="68" t="n"/>
-      <c r="K38" s="68" t="n"/>
-      <c r="L38" s="68" t="n"/>
-      <c r="M38" s="68" t="n"/>
-      <c r="N38" s="68" t="n"/>
-      <c r="O38" s="68" t="n"/>
-      <c r="P38" s="68" t="n"/>
-      <c r="Q38" s="68" t="n"/>
-      <c r="R38" s="68" t="n"/>
-      <c r="S38" s="68" t="n"/>
-      <c r="T38" s="68" t="n"/>
-      <c r="U38" s="68" t="n"/>
-      <c r="V38" s="68" t="n"/>
-      <c r="W38" s="68" t="n"/>
-      <c r="X38" s="68" t="n"/>
-    </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="B39" s="65" t="n"/>
-      <c r="C39" s="66" t="n"/>
-      <c r="D39" s="67" t="n"/>
-      <c r="E39" s="68" t="n"/>
-      <c r="F39" s="68" t="n"/>
-      <c r="G39" s="68" t="n"/>
-      <c r="H39" s="68" t="n"/>
-      <c r="I39" s="68" t="n"/>
-      <c r="J39" s="68" t="n"/>
-      <c r="K39" s="68" t="n"/>
-      <c r="L39" s="68" t="n"/>
-      <c r="M39" s="68" t="n"/>
-      <c r="N39" s="68" t="n"/>
-      <c r="O39" s="68" t="n"/>
-      <c r="P39" s="68" t="n"/>
-      <c r="Q39" s="68" t="n"/>
-      <c r="R39" s="68" t="n"/>
-      <c r="S39" s="68" t="n"/>
-      <c r="T39" s="68" t="n"/>
-      <c r="U39" s="68" t="n"/>
-      <c r="V39" s="68" t="n"/>
-      <c r="W39" s="68" t="n"/>
-      <c r="X39" s="68" t="n"/>
-    </row>
-    <row r="41" ht="21" customHeight="1">
-      <c r="B41" s="27" t="inlineStr">
-        <is>
-          <t>D  ·  THE CLINICIAN'S PLACE</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>D1 what they decide · D2 decide or advise · D3 adoption</t>
-        </is>
-      </c>
-      <c r="D42" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="B43" s="65" t="n"/>
-      <c r="C43" s="66" t="n"/>
-      <c r="D43" s="67" t="n"/>
-      <c r="E43" s="68" t="n"/>
-      <c r="F43" s="68" t="n"/>
-      <c r="G43" s="68" t="n"/>
-      <c r="H43" s="68" t="n"/>
-      <c r="I43" s="68" t="n"/>
-      <c r="J43" s="68" t="n"/>
-      <c r="K43" s="68" t="n"/>
-      <c r="L43" s="68" t="n"/>
-      <c r="M43" s="68" t="n"/>
-      <c r="N43" s="68" t="n"/>
-      <c r="O43" s="68" t="n"/>
-      <c r="P43" s="68" t="n"/>
-      <c r="Q43" s="68" t="n"/>
-      <c r="R43" s="68" t="n"/>
-      <c r="S43" s="68" t="n"/>
-      <c r="T43" s="68" t="n"/>
-      <c r="U43" s="68" t="n"/>
-      <c r="V43" s="68" t="n"/>
-      <c r="W43" s="68" t="n"/>
-      <c r="X43" s="68" t="n"/>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="B44" s="65" t="n"/>
-      <c r="C44" s="66" t="n"/>
-      <c r="D44" s="67" t="n"/>
-      <c r="E44" s="68" t="n"/>
-      <c r="F44" s="68" t="n"/>
-      <c r="G44" s="68" t="n"/>
-      <c r="H44" s="68" t="n"/>
-      <c r="I44" s="68" t="n"/>
-      <c r="J44" s="68" t="n"/>
-      <c r="K44" s="68" t="n"/>
-      <c r="L44" s="68" t="n"/>
-      <c r="M44" s="68" t="n"/>
-      <c r="N44" s="68" t="n"/>
-      <c r="O44" s="68" t="n"/>
-      <c r="P44" s="68" t="n"/>
-      <c r="Q44" s="68" t="n"/>
-      <c r="R44" s="68" t="n"/>
-      <c r="S44" s="68" t="n"/>
-      <c r="T44" s="68" t="n"/>
-      <c r="U44" s="68" t="n"/>
-      <c r="V44" s="68" t="n"/>
-      <c r="W44" s="68" t="n"/>
-      <c r="X44" s="68" t="n"/>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="B45" s="65" t="n"/>
-      <c r="C45" s="66" t="n"/>
-      <c r="D45" s="67" t="n"/>
-      <c r="E45" s="68" t="n"/>
-      <c r="F45" s="68" t="n"/>
-      <c r="G45" s="68" t="n"/>
-      <c r="H45" s="68" t="n"/>
-      <c r="I45" s="68" t="n"/>
-      <c r="J45" s="68" t="n"/>
-      <c r="K45" s="68" t="n"/>
-      <c r="L45" s="68" t="n"/>
-      <c r="M45" s="68" t="n"/>
-      <c r="N45" s="68" t="n"/>
-      <c r="O45" s="68" t="n"/>
-      <c r="P45" s="68" t="n"/>
-      <c r="Q45" s="68" t="n"/>
-      <c r="R45" s="68" t="n"/>
-      <c r="S45" s="68" t="n"/>
-      <c r="T45" s="68" t="n"/>
-      <c r="U45" s="68" t="n"/>
-      <c r="V45" s="68" t="n"/>
-      <c r="W45" s="68" t="n"/>
-      <c r="X45" s="68" t="n"/>
-    </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="B46" s="65" t="n"/>
-      <c r="C46" s="66" t="n"/>
-      <c r="D46" s="67" t="n"/>
-      <c r="E46" s="68" t="n"/>
-      <c r="F46" s="68" t="n"/>
-      <c r="G46" s="68" t="n"/>
-      <c r="H46" s="68" t="n"/>
-      <c r="I46" s="68" t="n"/>
-      <c r="J46" s="68" t="n"/>
-      <c r="K46" s="68" t="n"/>
-      <c r="L46" s="68" t="n"/>
-      <c r="M46" s="68" t="n"/>
-      <c r="N46" s="68" t="n"/>
-      <c r="O46" s="68" t="n"/>
-      <c r="P46" s="68" t="n"/>
-      <c r="Q46" s="68" t="n"/>
-      <c r="R46" s="68" t="n"/>
-      <c r="S46" s="68" t="n"/>
-      <c r="T46" s="68" t="n"/>
-      <c r="U46" s="68" t="n"/>
-      <c r="V46" s="68" t="n"/>
-      <c r="W46" s="68" t="n"/>
-      <c r="X46" s="68" t="n"/>
-    </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="B47" s="65" t="n"/>
-      <c r="C47" s="66" t="n"/>
-      <c r="D47" s="67" t="n"/>
-      <c r="E47" s="68" t="n"/>
-      <c r="F47" s="68" t="n"/>
-      <c r="G47" s="68" t="n"/>
-      <c r="H47" s="68" t="n"/>
-      <c r="I47" s="68" t="n"/>
-      <c r="J47" s="68" t="n"/>
-      <c r="K47" s="68" t="n"/>
-      <c r="L47" s="68" t="n"/>
-      <c r="M47" s="68" t="n"/>
-      <c r="N47" s="68" t="n"/>
-      <c r="O47" s="68" t="n"/>
-      <c r="P47" s="68" t="n"/>
-      <c r="Q47" s="68" t="n"/>
-      <c r="R47" s="68" t="n"/>
-      <c r="S47" s="68" t="n"/>
-      <c r="T47" s="68" t="n"/>
-      <c r="U47" s="68" t="n"/>
-      <c r="V47" s="68" t="n"/>
-      <c r="W47" s="68" t="n"/>
-      <c r="X47" s="68" t="n"/>
-    </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="B48" s="65" t="n"/>
-      <c r="C48" s="66" t="n"/>
-      <c r="D48" s="67" t="n"/>
-      <c r="E48" s="68" t="n"/>
-      <c r="F48" s="68" t="n"/>
-      <c r="G48" s="68" t="n"/>
-      <c r="H48" s="68" t="n"/>
-      <c r="I48" s="68" t="n"/>
-      <c r="J48" s="68" t="n"/>
-      <c r="K48" s="68" t="n"/>
-      <c r="L48" s="68" t="n"/>
-      <c r="M48" s="68" t="n"/>
-      <c r="N48" s="68" t="n"/>
-      <c r="O48" s="68" t="n"/>
-      <c r="P48" s="68" t="n"/>
-      <c r="Q48" s="68" t="n"/>
-      <c r="R48" s="68" t="n"/>
-      <c r="S48" s="68" t="n"/>
-      <c r="T48" s="68" t="n"/>
-      <c r="U48" s="68" t="n"/>
-      <c r="V48" s="68" t="n"/>
-      <c r="W48" s="68" t="n"/>
-      <c r="X48" s="68" t="n"/>
-    </row>
-    <row r="50" ht="21" customHeight="1">
-      <c r="B50" s="27" t="inlineStr">
-        <is>
-          <t>E  ·  FIT AND PARTNERSHIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>E1 what we did not ask · E2 sharing the value · E3 change management · E4 what they chose not to build</t>
-        </is>
-      </c>
-      <c r="D51" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="B52" s="65" t="n"/>
-      <c r="C52" s="66" t="n"/>
-      <c r="D52" s="67" t="n"/>
-      <c r="E52" s="68" t="n"/>
-      <c r="F52" s="68" t="n"/>
-      <c r="G52" s="68" t="n"/>
-      <c r="H52" s="68" t="n"/>
-      <c r="I52" s="68" t="n"/>
-      <c r="J52" s="68" t="n"/>
-      <c r="K52" s="68" t="n"/>
-      <c r="L52" s="68" t="n"/>
-      <c r="M52" s="68" t="n"/>
-      <c r="N52" s="68" t="n"/>
-      <c r="O52" s="68" t="n"/>
-      <c r="P52" s="68" t="n"/>
-      <c r="Q52" s="68" t="n"/>
-      <c r="R52" s="68" t="n"/>
-      <c r="S52" s="68" t="n"/>
-      <c r="T52" s="68" t="n"/>
-      <c r="U52" s="68" t="n"/>
-      <c r="V52" s="68" t="n"/>
-      <c r="W52" s="68" t="n"/>
-      <c r="X52" s="68" t="n"/>
-    </row>
-    <row r="53" ht="26" customHeight="1">
-      <c r="B53" s="65" t="n"/>
-      <c r="C53" s="66" t="n"/>
-      <c r="D53" s="67" t="n"/>
-      <c r="E53" s="68" t="n"/>
-      <c r="F53" s="68" t="n"/>
-      <c r="G53" s="68" t="n"/>
-      <c r="H53" s="68" t="n"/>
-      <c r="I53" s="68" t="n"/>
-      <c r="J53" s="68" t="n"/>
-      <c r="K53" s="68" t="n"/>
-      <c r="L53" s="68" t="n"/>
-      <c r="M53" s="68" t="n"/>
-      <c r="N53" s="68" t="n"/>
-      <c r="O53" s="68" t="n"/>
-      <c r="P53" s="68" t="n"/>
-      <c r="Q53" s="68" t="n"/>
-      <c r="R53" s="68" t="n"/>
-      <c r="S53" s="68" t="n"/>
-      <c r="T53" s="68" t="n"/>
-      <c r="U53" s="68" t="n"/>
-      <c r="V53" s="68" t="n"/>
-      <c r="W53" s="68" t="n"/>
-      <c r="X53" s="68" t="n"/>
-    </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="B54" s="65" t="n"/>
-      <c r="C54" s="66" t="n"/>
-      <c r="D54" s="67" t="n"/>
-      <c r="E54" s="68" t="n"/>
-      <c r="F54" s="68" t="n"/>
-      <c r="G54" s="68" t="n"/>
-      <c r="H54" s="68" t="n"/>
-      <c r="I54" s="68" t="n"/>
-      <c r="J54" s="68" t="n"/>
-      <c r="K54" s="68" t="n"/>
-      <c r="L54" s="68" t="n"/>
-      <c r="M54" s="68" t="n"/>
-      <c r="N54" s="68" t="n"/>
-      <c r="O54" s="68" t="n"/>
-      <c r="P54" s="68" t="n"/>
-      <c r="Q54" s="68" t="n"/>
-      <c r="R54" s="68" t="n"/>
-      <c r="S54" s="68" t="n"/>
-      <c r="T54" s="68" t="n"/>
-      <c r="U54" s="68" t="n"/>
-      <c r="V54" s="68" t="n"/>
-      <c r="W54" s="68" t="n"/>
-      <c r="X54" s="68" t="n"/>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="B55" s="65" t="n"/>
-      <c r="C55" s="66" t="n"/>
-      <c r="D55" s="67" t="n"/>
-      <c r="E55" s="68" t="n"/>
-      <c r="F55" s="68" t="n"/>
-      <c r="G55" s="68" t="n"/>
-      <c r="H55" s="68" t="n"/>
-      <c r="I55" s="68" t="n"/>
-      <c r="J55" s="68" t="n"/>
-      <c r="K55" s="68" t="n"/>
-      <c r="L55" s="68" t="n"/>
-      <c r="M55" s="68" t="n"/>
-      <c r="N55" s="68" t="n"/>
-      <c r="O55" s="68" t="n"/>
-      <c r="P55" s="68" t="n"/>
-      <c r="Q55" s="68" t="n"/>
-      <c r="R55" s="68" t="n"/>
-      <c r="S55" s="68" t="n"/>
-      <c r="T55" s="68" t="n"/>
-      <c r="U55" s="68" t="n"/>
-      <c r="V55" s="68" t="n"/>
-      <c r="W55" s="68" t="n"/>
-      <c r="X55" s="68" t="n"/>
-    </row>
-    <row r="56" ht="26" customHeight="1">
-      <c r="B56" s="65" t="n"/>
-      <c r="C56" s="66" t="n"/>
-      <c r="D56" s="67" t="n"/>
-      <c r="E56" s="68" t="n"/>
-      <c r="F56" s="68" t="n"/>
-      <c r="G56" s="68" t="n"/>
-      <c r="H56" s="68" t="n"/>
-      <c r="I56" s="68" t="n"/>
-      <c r="J56" s="68" t="n"/>
-      <c r="K56" s="68" t="n"/>
-      <c r="L56" s="68" t="n"/>
-      <c r="M56" s="68" t="n"/>
-      <c r="N56" s="68" t="n"/>
-      <c r="O56" s="68" t="n"/>
-      <c r="P56" s="68" t="n"/>
-      <c r="Q56" s="68" t="n"/>
-      <c r="R56" s="68" t="n"/>
-      <c r="S56" s="68" t="n"/>
-      <c r="T56" s="68" t="n"/>
-      <c r="U56" s="68" t="n"/>
-      <c r="V56" s="68" t="n"/>
-      <c r="W56" s="68" t="n"/>
-      <c r="X56" s="68" t="n"/>
-    </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="B57" s="65" t="n"/>
-      <c r="C57" s="66" t="n"/>
-      <c r="D57" s="67" t="n"/>
-      <c r="E57" s="68" t="n"/>
-      <c r="F57" s="68" t="n"/>
-      <c r="G57" s="68" t="n"/>
-      <c r="H57" s="68" t="n"/>
-      <c r="I57" s="68" t="n"/>
-      <c r="J57" s="68" t="n"/>
-      <c r="K57" s="68" t="n"/>
-      <c r="L57" s="68" t="n"/>
-      <c r="M57" s="68" t="n"/>
-      <c r="N57" s="68" t="n"/>
-      <c r="O57" s="68" t="n"/>
-      <c r="P57" s="68" t="n"/>
-      <c r="Q57" s="68" t="n"/>
-      <c r="R57" s="68" t="n"/>
-      <c r="S57" s="68" t="n"/>
-      <c r="T57" s="68" t="n"/>
-      <c r="U57" s="68" t="n"/>
-      <c r="V57" s="68" t="n"/>
-      <c r="W57" s="68" t="n"/>
-      <c r="X57" s="68" t="n"/>
-    </row>
-    <row r="59" ht="21" customHeight="1">
-      <c r="B59" s="27" t="inlineStr">
-        <is>
-          <t>INTANGIBLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Anything the feel section raised that a demo could settle</t>
-        </is>
-      </c>
-      <c r="D60" s="64" t="inlineStr">
-        <is>
-          <t>What would prove it</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="B61" s="65" t="n"/>
-      <c r="C61" s="66" t="n"/>
-      <c r="D61" s="67" t="n"/>
-      <c r="E61" s="68" t="n"/>
-      <c r="F61" s="68" t="n"/>
-      <c r="G61" s="68" t="n"/>
-      <c r="H61" s="68" t="n"/>
-      <c r="I61" s="68" t="n"/>
-      <c r="J61" s="68" t="n"/>
-      <c r="K61" s="68" t="n"/>
-      <c r="L61" s="68" t="n"/>
-      <c r="M61" s="68" t="n"/>
-      <c r="N61" s="68" t="n"/>
-      <c r="O61" s="68" t="n"/>
-      <c r="P61" s="68" t="n"/>
-      <c r="Q61" s="68" t="n"/>
-      <c r="R61" s="68" t="n"/>
-      <c r="S61" s="68" t="n"/>
-      <c r="T61" s="68" t="n"/>
-      <c r="U61" s="68" t="n"/>
-      <c r="V61" s="68" t="n"/>
-      <c r="W61" s="68" t="n"/>
-      <c r="X61" s="68" t="n"/>
-    </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="B62" s="65" t="n"/>
-      <c r="C62" s="66" t="n"/>
-      <c r="D62" s="67" t="n"/>
-      <c r="E62" s="68" t="n"/>
-      <c r="F62" s="68" t="n"/>
-      <c r="G62" s="68" t="n"/>
-      <c r="H62" s="68" t="n"/>
-      <c r="I62" s="68" t="n"/>
-      <c r="J62" s="68" t="n"/>
-      <c r="K62" s="68" t="n"/>
-      <c r="L62" s="68" t="n"/>
-      <c r="M62" s="68" t="n"/>
-      <c r="N62" s="68" t="n"/>
-      <c r="O62" s="68" t="n"/>
-      <c r="P62" s="68" t="n"/>
-      <c r="Q62" s="68" t="n"/>
-      <c r="R62" s="68" t="n"/>
-      <c r="S62" s="68" t="n"/>
-      <c r="T62" s="68" t="n"/>
-      <c r="U62" s="68" t="n"/>
-      <c r="V62" s="68" t="n"/>
-      <c r="W62" s="68" t="n"/>
-      <c r="X62" s="68" t="n"/>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="B63" s="65" t="n"/>
-      <c r="C63" s="66" t="n"/>
-      <c r="D63" s="67" t="n"/>
-      <c r="E63" s="68" t="n"/>
-      <c r="F63" s="68" t="n"/>
-      <c r="G63" s="68" t="n"/>
-      <c r="H63" s="68" t="n"/>
-      <c r="I63" s="68" t="n"/>
-      <c r="J63" s="68" t="n"/>
-      <c r="K63" s="68" t="n"/>
-      <c r="L63" s="68" t="n"/>
-      <c r="M63" s="68" t="n"/>
-      <c r="N63" s="68" t="n"/>
-      <c r="O63" s="68" t="n"/>
-      <c r="P63" s="68" t="n"/>
-      <c r="Q63" s="68" t="n"/>
-      <c r="R63" s="68" t="n"/>
-      <c r="S63" s="68" t="n"/>
-      <c r="T63" s="68" t="n"/>
-      <c r="U63" s="68" t="n"/>
-      <c r="V63" s="68" t="n"/>
-      <c r="W63" s="68" t="n"/>
-      <c r="X63" s="68" t="n"/>
-    </row>
-    <row r="64" ht="26" customHeight="1">
-      <c r="B64" s="65" t="n"/>
-      <c r="C64" s="66" t="n"/>
-      <c r="D64" s="67" t="n"/>
-      <c r="E64" s="68" t="n"/>
-      <c r="F64" s="68" t="n"/>
-      <c r="G64" s="68" t="n"/>
-      <c r="H64" s="68" t="n"/>
-      <c r="I64" s="68" t="n"/>
-      <c r="J64" s="68" t="n"/>
-      <c r="K64" s="68" t="n"/>
-      <c r="L64" s="68" t="n"/>
-      <c r="M64" s="68" t="n"/>
-      <c r="N64" s="68" t="n"/>
-      <c r="O64" s="68" t="n"/>
-      <c r="P64" s="68" t="n"/>
-      <c r="Q64" s="68" t="n"/>
-      <c r="R64" s="68" t="n"/>
-      <c r="S64" s="68" t="n"/>
-      <c r="T64" s="68" t="n"/>
-      <c r="U64" s="68" t="n"/>
-      <c r="V64" s="68" t="n"/>
-      <c r="W64" s="68" t="n"/>
-      <c r="X64" s="68" t="n"/>
-    </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="B65" s="65" t="n"/>
-      <c r="C65" s="66" t="n"/>
-      <c r="D65" s="67" t="n"/>
-      <c r="E65" s="68" t="n"/>
-      <c r="F65" s="68" t="n"/>
-      <c r="G65" s="68" t="n"/>
-      <c r="H65" s="68" t="n"/>
-      <c r="I65" s="68" t="n"/>
-      <c r="J65" s="68" t="n"/>
-      <c r="K65" s="68" t="n"/>
-      <c r="L65" s="68" t="n"/>
-      <c r="M65" s="68" t="n"/>
-      <c r="N65" s="68" t="n"/>
-      <c r="O65" s="68" t="n"/>
-      <c r="P65" s="68" t="n"/>
-      <c r="Q65" s="68" t="n"/>
-      <c r="R65" s="68" t="n"/>
-      <c r="S65" s="68" t="n"/>
-      <c r="T65" s="68" t="n"/>
-      <c r="U65" s="68" t="n"/>
-      <c r="V65" s="68" t="n"/>
-      <c r="W65" s="68" t="n"/>
-      <c r="X65" s="68" t="n"/>
-    </row>
-    <row r="66" ht="26" customHeight="1">
-      <c r="B66" s="65" t="n"/>
-      <c r="C66" s="66" t="n"/>
-      <c r="D66" s="67" t="n"/>
-      <c r="E66" s="68" t="n"/>
-      <c r="F66" s="68" t="n"/>
-      <c r="G66" s="68" t="n"/>
-      <c r="H66" s="68" t="n"/>
-      <c r="I66" s="68" t="n"/>
-      <c r="J66" s="68" t="n"/>
-      <c r="K66" s="68" t="n"/>
-      <c r="L66" s="68" t="n"/>
-      <c r="M66" s="68" t="n"/>
-      <c r="N66" s="68" t="n"/>
-      <c r="O66" s="68" t="n"/>
-      <c r="P66" s="68" t="n"/>
-      <c r="Q66" s="68" t="n"/>
-      <c r="R66" s="68" t="n"/>
-      <c r="S66" s="68" t="n"/>
-      <c r="T66" s="68" t="n"/>
-      <c r="U66" s="68" t="n"/>
-      <c r="V66" s="68" t="n"/>
-      <c r="W66" s="68" t="n"/>
-      <c r="X66" s="68" t="n"/>
+          <t>C  ·  HOW YOUR PRODUCT WORKS      C1 capacity · C2 assignment · C3 readiness · C4 the week · C5 recovery · C6 downtime · C7 the patient</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="B18" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="64" t="n"/>
+      <c r="E18" s="64" t="n"/>
+      <c r="F18" s="64" t="n"/>
+      <c r="G18" s="64" t="n"/>
+      <c r="H18" s="64" t="n"/>
+      <c r="I18" s="64" t="n"/>
+      <c r="J18" s="64" t="n"/>
+      <c r="K18" s="64" t="n"/>
+      <c r="L18" s="64" t="n"/>
+      <c r="M18" s="64" t="n"/>
+      <c r="N18" s="64" t="n"/>
+      <c r="O18" s="64" t="n"/>
+      <c r="P18" s="64" t="n"/>
+      <c r="Q18" s="64" t="n"/>
+      <c r="R18" s="64" t="n"/>
+      <c r="S18" s="64" t="n"/>
+      <c r="T18" s="64" t="n"/>
+      <c r="U18" s="64" t="n"/>
+      <c r="V18" s="64" t="n"/>
+      <c r="W18" s="64" t="n"/>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="B19" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="64" t="n"/>
+      <c r="E19" s="64" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="64" t="n"/>
+      <c r="I19" s="64" t="n"/>
+      <c r="J19" s="64" t="n"/>
+      <c r="K19" s="64" t="n"/>
+      <c r="L19" s="64" t="n"/>
+      <c r="M19" s="64" t="n"/>
+      <c r="N19" s="64" t="n"/>
+      <c r="O19" s="64" t="n"/>
+      <c r="P19" s="64" t="n"/>
+      <c r="Q19" s="64" t="n"/>
+      <c r="R19" s="64" t="n"/>
+      <c r="S19" s="64" t="n"/>
+      <c r="T19" s="64" t="n"/>
+      <c r="U19" s="64" t="n"/>
+      <c r="V19" s="64" t="n"/>
+      <c r="W19" s="64" t="n"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
+      <c r="B20" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="64" t="n"/>
+      <c r="I20" s="64" t="n"/>
+      <c r="J20" s="64" t="n"/>
+      <c r="K20" s="64" t="n"/>
+      <c r="L20" s="64" t="n"/>
+      <c r="M20" s="64" t="n"/>
+      <c r="N20" s="64" t="n"/>
+      <c r="O20" s="64" t="n"/>
+      <c r="P20" s="64" t="n"/>
+      <c r="Q20" s="64" t="n"/>
+      <c r="R20" s="64" t="n"/>
+      <c r="S20" s="64" t="n"/>
+      <c r="T20" s="64" t="n"/>
+      <c r="U20" s="64" t="n"/>
+      <c r="V20" s="64" t="n"/>
+      <c r="W20" s="64" t="n"/>
+    </row>
+    <row r="22" ht="21" customHeight="1">
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>D  ·  THE CLINICIAN'S PLACE      D1 what they decide · D2 decide or advise · D3 adoption</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46" customHeight="1">
+      <c r="B23" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="64" t="n"/>
+      <c r="E23" s="64" t="n"/>
+      <c r="F23" s="64" t="n"/>
+      <c r="G23" s="64" t="n"/>
+      <c r="H23" s="64" t="n"/>
+      <c r="I23" s="64" t="n"/>
+      <c r="J23" s="64" t="n"/>
+      <c r="K23" s="64" t="n"/>
+      <c r="L23" s="64" t="n"/>
+      <c r="M23" s="64" t="n"/>
+      <c r="N23" s="64" t="n"/>
+      <c r="O23" s="64" t="n"/>
+      <c r="P23" s="64" t="n"/>
+      <c r="Q23" s="64" t="n"/>
+      <c r="R23" s="64" t="n"/>
+      <c r="S23" s="64" t="n"/>
+      <c r="T23" s="64" t="n"/>
+      <c r="U23" s="64" t="n"/>
+      <c r="V23" s="64" t="n"/>
+      <c r="W23" s="64" t="n"/>
+    </row>
+    <row r="24" ht="46" customHeight="1">
+      <c r="B24" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="64" t="n"/>
+      <c r="E24" s="64" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="64" t="n"/>
+      <c r="H24" s="64" t="n"/>
+      <c r="I24" s="64" t="n"/>
+      <c r="J24" s="64" t="n"/>
+      <c r="K24" s="64" t="n"/>
+      <c r="L24" s="64" t="n"/>
+      <c r="M24" s="64" t="n"/>
+      <c r="N24" s="64" t="n"/>
+      <c r="O24" s="64" t="n"/>
+      <c r="P24" s="64" t="n"/>
+      <c r="Q24" s="64" t="n"/>
+      <c r="R24" s="64" t="n"/>
+      <c r="S24" s="64" t="n"/>
+      <c r="T24" s="64" t="n"/>
+      <c r="U24" s="64" t="n"/>
+      <c r="V24" s="64" t="n"/>
+      <c r="W24" s="64" t="n"/>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="B25" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="64" t="n"/>
+      <c r="E25" s="64" t="n"/>
+      <c r="F25" s="64" t="n"/>
+      <c r="G25" s="64" t="n"/>
+      <c r="H25" s="64" t="n"/>
+      <c r="I25" s="64" t="n"/>
+      <c r="J25" s="64" t="n"/>
+      <c r="K25" s="64" t="n"/>
+      <c r="L25" s="64" t="n"/>
+      <c r="M25" s="64" t="n"/>
+      <c r="N25" s="64" t="n"/>
+      <c r="O25" s="64" t="n"/>
+      <c r="P25" s="64" t="n"/>
+      <c r="Q25" s="64" t="n"/>
+      <c r="R25" s="64" t="n"/>
+      <c r="S25" s="64" t="n"/>
+      <c r="T25" s="64" t="n"/>
+      <c r="U25" s="64" t="n"/>
+      <c r="V25" s="64" t="n"/>
+      <c r="W25" s="64" t="n"/>
+    </row>
+    <row r="27" ht="21" customHeight="1">
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>E  ·  FIT AND PARTNERSHIP      E1 what we did not ask · E2 sharing the value · E3 change management · E4 what they chose not to build</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="46" customHeight="1">
+      <c r="B28" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="64" t="n"/>
+      <c r="E28" s="64" t="n"/>
+      <c r="F28" s="64" t="n"/>
+      <c r="G28" s="64" t="n"/>
+      <c r="H28" s="64" t="n"/>
+      <c r="I28" s="64" t="n"/>
+      <c r="J28" s="64" t="n"/>
+      <c r="K28" s="64" t="n"/>
+      <c r="L28" s="64" t="n"/>
+      <c r="M28" s="64" t="n"/>
+      <c r="N28" s="64" t="n"/>
+      <c r="O28" s="64" t="n"/>
+      <c r="P28" s="64" t="n"/>
+      <c r="Q28" s="64" t="n"/>
+      <c r="R28" s="64" t="n"/>
+      <c r="S28" s="64" t="n"/>
+      <c r="T28" s="64" t="n"/>
+      <c r="U28" s="64" t="n"/>
+      <c r="V28" s="64" t="n"/>
+      <c r="W28" s="64" t="n"/>
+    </row>
+    <row r="29" ht="46" customHeight="1">
+      <c r="B29" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="64" t="n"/>
+      <c r="E29" s="64" t="n"/>
+      <c r="F29" s="64" t="n"/>
+      <c r="G29" s="64" t="n"/>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="64" t="n"/>
+      <c r="J29" s="64" t="n"/>
+      <c r="K29" s="64" t="n"/>
+      <c r="L29" s="64" t="n"/>
+      <c r="M29" s="64" t="n"/>
+      <c r="N29" s="64" t="n"/>
+      <c r="O29" s="64" t="n"/>
+      <c r="P29" s="64" t="n"/>
+      <c r="Q29" s="64" t="n"/>
+      <c r="R29" s="64" t="n"/>
+      <c r="S29" s="64" t="n"/>
+      <c r="T29" s="64" t="n"/>
+      <c r="U29" s="64" t="n"/>
+      <c r="V29" s="64" t="n"/>
+      <c r="W29" s="64" t="n"/>
+    </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="B30" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="64" t="n"/>
+      <c r="E30" s="64" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="64" t="n"/>
+      <c r="J30" s="64" t="n"/>
+      <c r="K30" s="64" t="n"/>
+      <c r="L30" s="64" t="n"/>
+      <c r="M30" s="64" t="n"/>
+      <c r="N30" s="64" t="n"/>
+      <c r="O30" s="64" t="n"/>
+      <c r="P30" s="64" t="n"/>
+      <c r="Q30" s="64" t="n"/>
+      <c r="R30" s="64" t="n"/>
+      <c r="S30" s="64" t="n"/>
+      <c r="T30" s="64" t="n"/>
+      <c r="U30" s="64" t="n"/>
+      <c r="V30" s="64" t="n"/>
+      <c r="W30" s="64" t="n"/>
+    </row>
+    <row r="32" ht="21" customHeight="1">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>INTANGIBLES      anything the feel section raised that a demo could settle</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="46" customHeight="1">
+      <c r="B33" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="64" t="n"/>
+      <c r="E33" s="64" t="n"/>
+      <c r="F33" s="64" t="n"/>
+      <c r="G33" s="64" t="n"/>
+      <c r="H33" s="64" t="n"/>
+      <c r="I33" s="64" t="n"/>
+      <c r="J33" s="64" t="n"/>
+      <c r="K33" s="64" t="n"/>
+      <c r="L33" s="64" t="n"/>
+      <c r="M33" s="64" t="n"/>
+      <c r="N33" s="64" t="n"/>
+      <c r="O33" s="64" t="n"/>
+      <c r="P33" s="64" t="n"/>
+      <c r="Q33" s="64" t="n"/>
+      <c r="R33" s="64" t="n"/>
+      <c r="S33" s="64" t="n"/>
+      <c r="T33" s="64" t="n"/>
+      <c r="U33" s="64" t="n"/>
+      <c r="V33" s="64" t="n"/>
+      <c r="W33" s="64" t="n"/>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="B34" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="64" t="n"/>
+      <c r="E34" s="64" t="n"/>
+      <c r="F34" s="64" t="n"/>
+      <c r="G34" s="64" t="n"/>
+      <c r="H34" s="64" t="n"/>
+      <c r="I34" s="64" t="n"/>
+      <c r="J34" s="64" t="n"/>
+      <c r="K34" s="64" t="n"/>
+      <c r="L34" s="64" t="n"/>
+      <c r="M34" s="64" t="n"/>
+      <c r="N34" s="64" t="n"/>
+      <c r="O34" s="64" t="n"/>
+      <c r="P34" s="64" t="n"/>
+      <c r="Q34" s="64" t="n"/>
+      <c r="R34" s="64" t="n"/>
+      <c r="S34" s="64" t="n"/>
+      <c r="T34" s="64" t="n"/>
+      <c r="U34" s="64" t="n"/>
+      <c r="V34" s="64" t="n"/>
+      <c r="W34" s="64" t="n"/>
+    </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="B35" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="64" t="n"/>
+      <c r="E35" s="64" t="n"/>
+      <c r="F35" s="64" t="n"/>
+      <c r="G35" s="64" t="n"/>
+      <c r="H35" s="64" t="n"/>
+      <c r="I35" s="64" t="n"/>
+      <c r="J35" s="64" t="n"/>
+      <c r="K35" s="64" t="n"/>
+      <c r="L35" s="64" t="n"/>
+      <c r="M35" s="64" t="n"/>
+      <c r="N35" s="64" t="n"/>
+      <c r="O35" s="64" t="n"/>
+      <c r="P35" s="64" t="n"/>
+      <c r="Q35" s="64" t="n"/>
+      <c r="R35" s="64" t="n"/>
+      <c r="S35" s="64" t="n"/>
+      <c r="T35" s="64" t="n"/>
+      <c r="U35" s="64" t="n"/>
+      <c r="V35" s="64" t="n"/>
+      <c r="W35" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B17:X17"/>
-    <mergeCell ref="B41:X41"/>
-    <mergeCell ref="B8:X8"/>
-    <mergeCell ref="B4:X4"/>
-    <mergeCell ref="B50:X50"/>
-    <mergeCell ref="B59:X59"/>
-    <mergeCell ref="B28:X28"/>
+    <mergeCell ref="B3:W3"/>
+    <mergeCell ref="B27:W27"/>
+    <mergeCell ref="B22:W22"/>
+    <mergeCell ref="B32:W32"/>
+    <mergeCell ref="B17:W17"/>
+    <mergeCell ref="B12:W12"/>
+    <mergeCell ref="B7:W7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 

</xml_diff>